<commit_message>
Revisão de código e refatorações
- Melhorando o fluxo com Langgraph
- Reasoning a nivel de agente
- Adicionando HIL para tomada de decisão
- Melhorando mensagens e logs
</commit_message>
<xml_diff>
--- a/files/avaliações.xlsx
+++ b/files/avaliações.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\gestor-avaliacoes\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\gestor_avaliacoes_performance\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46E3ECC-7F0D-4424-87E7-112540060D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97D9D5D9-4049-4482-8A71-BA6973520BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -78,9 +78,6 @@
     <t>RH</t>
   </si>
   <si>
-    <t>Elena Rose</t>
-  </si>
-  <si>
     <t>Financeiro</t>
   </si>
   <si>
@@ -96,7 +93,10 @@
     <t>Psicólogo</t>
   </si>
   <si>
-    <t>Analista de pagamentos</t>
+    <t>Auxiliar Administrativo</t>
+  </si>
+  <si>
+    <t>Roberta Vieira</t>
   </si>
 </sst>
 </file>
@@ -104,7 +104,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -165,16 +165,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,10 +456,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" customWidth="1"/>
     <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -468,7 +469,7 @@
     <col min="8" max="8" width="8.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,25 +500,25 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="4">
         <f>AVERAGE(E2:H2)</f>
         <v>4.8</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>5</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>4.5</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="4">
         <v>4.7</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
         <v>5</v>
       </c>
     </row>
@@ -526,25 +527,25 @@
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3">
-        <f t="shared" ref="D3:D6" si="0">AVERAGE(E3:H3)</f>
+      <c r="D3" s="4">
+        <f t="shared" ref="D3:D5" si="0">AVERAGE(E3:H3)</f>
         <v>4.55</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>4.9000000000000004</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>5</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>4.8</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
         <v>3.5</v>
       </c>
     </row>
@@ -553,25 +554,25 @@
         <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="4">
         <f t="shared" si="0"/>
         <v>4.25</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>3.5</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="4">
         <v>4</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>4.5</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
         <v>5</v>
       </c>
     </row>
@@ -580,54 +581,57 @@
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="4">
         <f t="shared" si="0"/>
         <v>3.15</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="4">
         <v>3</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="4">
         <v>3.5</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="4">
         <v>3</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="4">
         <v>3.1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="D6" s="4">
         <f>AVERAGE(E6:H6)</f>
-        <v>4.4749999999999996</v>
-      </c>
-      <c r="E6" s="3">
-        <v>5</v>
-      </c>
-      <c r="F6" s="3">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="G6" s="3">
-        <v>4.3</v>
-      </c>
-      <c r="H6" s="3">
-        <v>4.2</v>
-      </c>
+        <v>4.5</v>
+      </c>
+      <c r="E6" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="F6" s="4">
+        <v>4.7</v>
+      </c>
+      <c r="G6" s="4">
+        <v>4.8</v>
+      </c>
+      <c r="H6" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>